<commit_message>
Pre-fill each lab workbook's Prompt_Log with the lab's prompts
Prompt_Log now lists every step prompt (Step, Mode, Prompt) plus the extra
sample prompts, parsed by the shared lab_prompts.py so the workbook and the
prompts page always match. Copilot fills What Copilot did, How I verified
and Decision. Check formulas move to a Checks sheet. Data sheets unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
+++ b/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
@@ -68,7 +68,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -78,6 +78,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -14232,12 +14235,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
@@ -14275,7 +14278,371 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>2 · A</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>Format the data on the Applications sheet (from A1 to the last row and column) as an Excel table with headers. Name the table tblApplications. Do not change, sort or delete any values. Then tell me the table name, the number of columns and the number of data rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>3 · B</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>GOAL: Describe this candidate pipeline before I analyse it.
+CONTEXT: BrightPath recruitment desk, H1 2026. One row should be one application.
+DATA: Use only tblApplications.
+CONSTRAINTS: Do not change the workbook.
+OUTPUT: What a row represents, each column with its data type, the number of rows, the Applied_Date range and the distinct values of Stage and Source.
+REVIEW: Tell me how you counted the rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>4 · C</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Check tblApplications for data-quality issues. List any Application_ID that appears more than once, and any Source value that is not exactly one of: LinkedIn, JobStreet, MyCareersFuture, Referral, BrightPath Website, Job Fair, Talent Database. Give the count of each issue. Do not change anything.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>4 · D</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>1) Highlight Application_ID cells that appear more than once in tblApplications with an orange fill.
+2) Add a column Source_Clean to tblApplications that trims spaces from Source and changes 'Linked In' to 'LinkedIn'. Do not delete or edit any existing values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>5 · E</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean. Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>5 · F</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>On a sheet named Checks (create it if needed), add these formulas with a label beside each, then tell me the results:
+=COUNTIFS(tblApplications[Stage],"Hired")
+=COUNTIFS(tblApplications[Source_Clean],"LinkedIn",tblApplications[Stage],"Hired")</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>6 · G</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>6 · H</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>6 · I</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>6 · J</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>How many rows of tblApplications are visible with this filter?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>6 · K</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>7 · L</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Extra 1</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Extra 2</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Extra 3</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Extra 4</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Extra 5</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Extra 6</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Highlight rows where Stage is Hired in light green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Extra 7</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Extra 8</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Filter to show only Technology applications at the Interview stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Extra 9</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>What's interesting about this pipeline data? Give three observations, each with the numbers behind it.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Lab 1: point to the Source fix and verify Source_Clean after it
Step 3 tells learners that Source label issues Copilot spots are fixed in
Step 4; a follow-up after Prompt D lists Source_Clean values to confirm the
fix and that all 242 rows remain.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
+++ b/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
@@ -14235,7 +14235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14355,17 +14355,17 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>5 · E</t>
+          <t>4 · E</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean. Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+          <t>List the distinct Source_Clean values with a count of each. Confirm there is no 'Linked In' and no value with a trailing space, and that tblApplications still has 242 rows.</t>
         </is>
       </c>
     </row>
@@ -14377,10 +14377,27 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean. Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>5 · G</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
           <t>Edit</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>On a sheet named Checks (create it if needed), add these formulas with a label beside each, then tell me the results:
 =COUNTIFS(tblApplications[Stage],"Hired")
@@ -14388,23 +14405,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>6 · G</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Edit</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
@@ -14418,7 +14418,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14435,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
         </is>
       </c>
     </row>
@@ -14452,7 +14452,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>How many rows of tblApplications are visible with this filter?</t>
+          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
         </is>
       </c>
     </row>
@@ -14469,14 +14469,14 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
+          <t>How many rows of tblApplications are visible with this filter?</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>7 · L</t>
+          <t>6 · L</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -14486,31 +14486,31 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
+          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Extra 1</t>
+          <t>7 · M</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
+          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Extra 2</t>
+          <t>Extra 1</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -14520,14 +14520,14 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
+          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Extra 3</t>
+          <t>Extra 2</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
@@ -14537,14 +14537,14 @@
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
+          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Extra 4</t>
+          <t>Extra 3</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -14554,14 +14554,14 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
+          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Extra 5</t>
+          <t>Extra 4</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14571,14 +14571,14 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
+          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Extra 6</t>
+          <t>Extra 5</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -14588,14 +14588,14 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Highlight rows where Stage is Hired in light green.</t>
+          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Extra 7</t>
+          <t>Extra 6</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14605,14 +14605,14 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+          <t>Highlight rows where Stage is Hired in light green.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Extra 8</t>
+          <t>Extra 7</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -14622,22 +14622,39 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Filter to show only Technology applications at the Interview stage.</t>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
+          <t>Extra 8</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Filter to show only Technology applications at the Interview stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
           <t>Extra 9</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Any</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>What's interesting about this pipeline data? Give three observations, each with the numbers behind it.</t>
         </is>

</xml_diff>

<commit_message>
Lab 1: highlight the Source cells that Source_Clean fixed (yellow)
New follow-up after the Source_Clean prompt highlights the 5 Source cells
whose label was cleaned ('Linked In' x3, 'JobStreet ' x2) and lists their
IDs; Test It expects 5 yellow cells. Rebuilt Lab 1 files and the prompts page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
+++ b/labs/lab-01-explore-and-question-recruitment-pipeline-data/data/BrightPath_Candidate_Pipeline.xlsx
@@ -14235,7 +14235,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14365,31 +14365,31 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>List the distinct Source_Clean values with a count of each. Confirm there is no 'Linked In' and no value with a trailing space, and that tblApplications still has 242 rows.</t>
+          <t>For each duplicated Application_ID, give the row numbers of both copies and say whether the two rows are identical.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>5 · F</t>
+          <t>4 · F</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Chat</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean. Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+          <t>Highlight the Source cells in tblApplications where Source_Clean is different from Source with a yellow fill. Tell me how many cells you highlighted and list their Application_IDs.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>5 · G</t>
+          <t>4 · G</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -14398,6 +14398,40 @@
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>List the distinct Source_Clean values with a count of each. Confirm there is no 'Linked In' and no value with a trailing space, and that tblApplications still has 242 rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>5 · H</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Chat</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Using tblApplications, count applications and hires (Stage = "Hired") by Source_Clean. Show a table sorted by hires, highest first, with hire rate = hires / applications.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>5 · I</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Edit</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>On a sheet named Checks (create it if needed), add these formulas with a label beside each, then tell me the results:
 =COUNTIFS(tblApplications[Stage],"Hired")
@@ -14405,40 +14439,6 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>6 · H</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Edit</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>6 · I</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Edit</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -14452,7 +14452,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
+          <t>Highlight entire rows of tblApplications where Stage is "Hired" with a light green fill.</t>
         </is>
       </c>
     </row>
@@ -14469,7 +14469,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>How many rows of tblApplications are visible with this filter?</t>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
         </is>
       </c>
     </row>
@@ -14486,14 +14486,14 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
+          <t>Filter tblApplications to show only Client_Sector = "Technology" and Stage = "Interview".</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>7 · M</t>
+          <t>6 · M</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -14503,48 +14503,48 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
+          <t>How many rows of tblApplications are visible with this filter?</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Extra 1</t>
+          <t>6 · N</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
+          <t>Clear all filters on tblApplications and confirm all 242 rows are visible.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Extra 2</t>
+          <t>7 · O</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>Any</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
+          <t>Prompt_Log already lists every prompt in this lab. For each one I ran, fill in What Copilot did and How I verified, and set Decision to Keep. I will tell you any row to change to Revise or Undo.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Extra 3</t>
+          <t>Extra 1</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
@@ -14554,14 +14554,14 @@
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
+          <t>Describe tblApplications: what one row represents, each column's data type, the row count and the Applied_Date range. Do not change the workbook.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Extra 4</t>
+          <t>Extra 2</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
@@ -14571,14 +14571,14 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
+          <t>List any Application_ID that appears more than once in tblApplications and any Source value that is not in the canonical list on About_This_Data.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>Extra 5</t>
+          <t>Extra 3</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -14588,14 +14588,14 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
+          <t>Add a column Source_Clean that trims spaces from Source and replaces 'Linked In' with 'LinkedIn'. Do not change the original Source column.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Extra 6</t>
+          <t>Extra 4</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
@@ -14605,14 +14605,14 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Highlight rows where Stage is Hired in light green.</t>
+          <t>Using tblApplications, count applications and hires by Source_Clean and show the hire rate. Sort by hires, highest first.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>Extra 7</t>
+          <t>Extra 5</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
@@ -14622,14 +14622,14 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+          <t>Which Client_Sector received the most applications, and how many? Show the count for every sector.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Extra 8</t>
+          <t>Extra 6</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
@@ -14639,22 +14639,56 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Filter to show only Technology applications at the Interview stage.</t>
+          <t>Highlight rows where Stage is Hired in light green.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
+          <t>Extra 7</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Sort tblApplications by Interview_Score from highest to lowest, then by Days_in_Pipeline from lowest to highest.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Extra 8</t>
+        </is>
+      </c>
+      <c r="B24" s="7" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Filter to show only Technology applications at the Interview stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
           <t>Extra 9</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Any</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>What's interesting about this pipeline data? Give three observations, each with the numbers behind it.</t>
         </is>

</xml_diff>